<commit_message>
chore: monthly retrain (2026-08-01)
</commit_message>
<xml_diff>
--- a/wsts_historical.xlsx
+++ b/wsts_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpwsts-my.sharepoint.com/personal/admin_tpwsts_onmicrosoft_com/Documents/WSTS/2-WSTS-Statistic-Reports/Blue Book/Blue Book 2026/BB-04-26/BB-04-26-final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpwsts-my.sharepoint.com/personal/admin_tpwsts_onmicrosoft_com/Documents/WSTS/2-WSTS-Statistic-Reports/Blue Book/Blue Book 2026/BB-05-26/BB-05-26-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="45" documentId="13_ncr:1_{95B6A9BD-11A5-4993-BD56-443C8CBE0F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D9A45AF1-3CE6-4FBB-8E4C-CA54551C8938}"/>
+  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{95B6A9BD-11A5-4993-BD56-443C8CBE0F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71467896-B56F-4B60-BBEC-8A86FB4242E2}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Data" sheetId="1" r:id="rId1"/>
@@ -913,19 +913,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R250"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.77734375" style="7" customWidth="1"/>
-    <col min="2" max="2" width="10.33203125" customWidth="1"/>
-    <col min="3" max="9" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="10.33203125" customWidth="1"/>
-    <col min="14" max="14" width="11.44140625" style="7" customWidth="1"/>
-    <col min="15" max="18" width="11.109375" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.75" style="7" customWidth="1"/>
+    <col min="2" max="2" width="10.375" customWidth="1"/>
+    <col min="3" max="9" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.5" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.375" customWidth="1"/>
+    <col min="14" max="14" width="11.5" style="7" customWidth="1"/>
+    <col min="15" max="18" width="11.125" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -933,7 +933,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="18" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -14293,7 +14293,9 @@
       <c r="E246" s="6">
         <v>41534424</v>
       </c>
-      <c r="F246" s="6"/>
+      <c r="F246" s="6">
+        <v>46422927</v>
+      </c>
       <c r="G246" s="6"/>
       <c r="H246" s="6"/>
       <c r="I246" s="6"/>
@@ -14303,7 +14305,7 @@
       <c r="M246" s="5"/>
       <c r="N246" s="8">
         <f>SUM(B246:M246)</f>
-        <v>142955084</v>
+        <v>189378011</v>
       </c>
       <c r="O246" s="11">
         <f>SUM(B246:D246)</f>
@@ -14311,7 +14313,7 @@
       </c>
       <c r="P246" s="11">
         <f>SUM(E246:G246)</f>
-        <v>41534424</v>
+        <v>87957351</v>
       </c>
       <c r="Q246" s="11">
         <f>SUM(H246:J246)</f>
@@ -14338,7 +14340,9 @@
       <c r="E247" s="6">
         <v>6754705</v>
       </c>
-      <c r="F247" s="6"/>
+      <c r="F247" s="6">
+        <v>8014839</v>
+      </c>
       <c r="G247" s="6"/>
       <c r="H247" s="6"/>
       <c r="I247" s="6"/>
@@ -14348,7 +14352,7 @@
       <c r="M247" s="5"/>
       <c r="N247" s="8">
         <f>SUM(B247:M247)</f>
-        <v>25352589</v>
+        <v>33367428</v>
       </c>
       <c r="O247" s="11">
         <f>SUM(B247:D247)</f>
@@ -14356,7 +14360,7 @@
       </c>
       <c r="P247" s="11">
         <f>SUM(E247:G247)</f>
-        <v>6754705</v>
+        <v>14769544</v>
       </c>
       <c r="Q247" s="11">
         <f>SUM(H247:J247)</f>
@@ -14383,7 +14387,9 @@
       <c r="E248" s="6">
         <v>4428604</v>
       </c>
-      <c r="F248" s="6"/>
+      <c r="F248" s="6">
+        <v>4857631</v>
+      </c>
       <c r="G248" s="6"/>
       <c r="H248" s="6"/>
       <c r="I248" s="6"/>
@@ -14393,7 +14399,7 @@
       <c r="M248" s="5"/>
       <c r="N248" s="8">
         <f>SUM(B248:M248)</f>
-        <v>16578623</v>
+        <v>21436254</v>
       </c>
       <c r="O248" s="11">
         <f>SUM(B248:D248)</f>
@@ -14401,7 +14407,7 @@
       </c>
       <c r="P248" s="11">
         <f>SUM(E248:G248)</f>
-        <v>4428604</v>
+        <v>9286235</v>
       </c>
       <c r="Q248" s="11">
         <f>SUM(H248:J248)</f>
@@ -14428,7 +14434,9 @@
       <c r="E249" s="6">
         <v>60958983</v>
       </c>
-      <c r="F249" s="6"/>
+      <c r="F249" s="6">
+        <v>72642332</v>
+      </c>
       <c r="G249" s="6"/>
       <c r="H249" s="6"/>
       <c r="I249" s="6"/>
@@ -14438,7 +14446,7 @@
       <c r="M249" s="5"/>
       <c r="N249" s="8">
         <f>SUM(B249:M249)</f>
-        <v>227336052</v>
+        <v>299978384</v>
       </c>
       <c r="O249" s="11">
         <f>SUM(B249:D249)</f>
@@ -14446,7 +14454,7 @@
       </c>
       <c r="P249" s="11">
         <f>SUM(E249:G249)</f>
-        <v>60958983</v>
+        <v>133601315</v>
       </c>
       <c r="Q249" s="11">
         <f>SUM(H249:J249)</f>
@@ -14473,7 +14481,9 @@
       <c r="E250" s="6">
         <v>113676716</v>
       </c>
-      <c r="F250" s="6"/>
+      <c r="F250" s="6">
+        <v>131937729</v>
+      </c>
       <c r="G250" s="6"/>
       <c r="H250" s="6"/>
       <c r="I250" s="6"/>
@@ -14483,7 +14493,7 @@
       <c r="M250" s="5"/>
       <c r="N250" s="8">
         <f>SUM(N246:N249)</f>
-        <v>412222348</v>
+        <v>544160077</v>
       </c>
       <c r="O250" s="11">
         <f>SUM(B250:D250)</f>
@@ -14491,7 +14501,7 @@
       </c>
       <c r="P250" s="11">
         <f>SUM(E250:G250)</f>
-        <v>113676716</v>
+        <v>245614445</v>
       </c>
       <c r="Q250" s="11">
         <f>SUM(H250:J250)</f>
@@ -14586,18 +14596,18 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M250"/>
-  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.33203125" customWidth="1"/>
-    <col min="2" max="4" width="10.33203125" customWidth="1"/>
-    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="13" width="10.33203125" customWidth="1"/>
-    <col min="14" max="17" width="9.33203125" customWidth="1"/>
-    <col min="18" max="18" width="3.77734375" customWidth="1"/>
-    <col min="19" max="19" width="5.109375" customWidth="1"/>
+    <col min="1" max="1" width="18.375" customWidth="1"/>
+    <col min="2" max="4" width="10.375" customWidth="1"/>
+    <col min="5" max="5" width="11.125" bestFit="1" customWidth="1"/>
+    <col min="6" max="13" width="10.375" customWidth="1"/>
+    <col min="14" max="17" width="9.375" customWidth="1"/>
+    <col min="18" max="18" width="3.75" customWidth="1"/>
+    <col min="19" max="19" width="5.125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.4">
+    <row r="1" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -14605,14 +14615,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.4">
+    <row r="2" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="F2" s="1"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -24718,7 +24728,7 @@
       </c>
       <c r="F246" s="5">
         <f>IF('Monthly Data'!F246=0,0,AVERAGE('Monthly Data'!D246,'Monthly Data'!E246,'Monthly Data'!F246))</f>
-        <v>0</v>
+        <v>42851068.333333336</v>
       </c>
       <c r="G246" s="5">
         <f>IF('Monthly Data'!G246=0,0,AVERAGE('Monthly Data'!E246,'Monthly Data'!F246,'Monthly Data'!G246))</f>
@@ -24771,7 +24781,7 @@
       </c>
       <c r="F247" s="5">
         <f>IF('Monthly Data'!F247=0,0,AVERAGE('Monthly Data'!D247,'Monthly Data'!E247,'Monthly Data'!F247))</f>
-        <v>0</v>
+        <v>7100167.666666667</v>
       </c>
       <c r="G247" s="5">
         <f>IF('Monthly Data'!G247=0,0,AVERAGE('Monthly Data'!E247,'Monthly Data'!F247,'Monthly Data'!G247))</f>
@@ -24824,7 +24834,7 @@
       </c>
       <c r="F248" s="5">
         <f>IF('Monthly Data'!F248=0,0,AVERAGE('Monthly Data'!D248,'Monthly Data'!E248,'Monthly Data'!F248))</f>
-        <v>0</v>
+        <v>4584509</v>
       </c>
       <c r="G248" s="5">
         <f>IF('Monthly Data'!G248=0,0,AVERAGE('Monthly Data'!E248,'Monthly Data'!F248,'Monthly Data'!G248))</f>
@@ -24877,7 +24887,7 @@
       </c>
       <c r="F249" s="5">
         <f>IF('Monthly Data'!F249=0,0,AVERAGE('Monthly Data'!D249,'Monthly Data'!E249,'Monthly Data'!F249))</f>
-        <v>0</v>
+        <v>66072269</v>
       </c>
       <c r="G249" s="5">
         <f>IF('Monthly Data'!G249=0,0,AVERAGE('Monthly Data'!E249,'Monthly Data'!F249,'Monthly Data'!G249))</f>
@@ -24930,7 +24940,7 @@
       </c>
       <c r="F250" s="5">
         <f>IF('Monthly Data'!F250=0,0,AVERAGE('Monthly Data'!D250,'Monthly Data'!E250,'Monthly Data'!F250))</f>
-        <v>0</v>
+        <v>120608014</v>
       </c>
       <c r="G250" s="5">
         <f>IF('Monthly Data'!G250=0,0,AVERAGE('Monthly Data'!E250,'Monthly Data'!F250,'Monthly Data'!G250))</f>

</xml_diff>

<commit_message>
chore: monthly retrain (2026-09-01)
</commit_message>
<xml_diff>
--- a/wsts_historical.xlsx
+++ b/wsts_historical.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpwsts-my.sharepoint.com/personal/admin_tpwsts_onmicrosoft_com/Documents/WSTS/2-WSTS-Statistic-Reports/Blue Book/Blue Book 2026/BB-05-26/BB-05-26-final/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://tpwsts-my.sharepoint.com/personal/admin_tpwsts_onmicrosoft_com/Documents/WSTS/2-WSTS-Statistic-Reports/Blue Book/Blue Book 2026/BB-06-26/BB-ß6-26-final/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="46" documentId="13_ncr:1_{95B6A9BD-11A5-4993-BD56-443C8CBE0F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{71467896-B56F-4B60-BBEC-8A86FB4242E2}"/>
+  <xr:revisionPtr revIDLastSave="52" documentId="13_ncr:1_{95B6A9BD-11A5-4993-BD56-443C8CBE0F5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{27B4020C-B8F3-477B-BA71-2C0A556FC1C0}"/>
   <bookViews>
-    <workbookView xWindow="30612" yWindow="-108" windowWidth="30936" windowHeight="16776" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="24220" windowHeight="15500" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Monthly Data" sheetId="1" r:id="rId1"/>
@@ -557,7 +557,7 @@
     </xdr:from>
     <xdr:to>
       <xdr:col>12</xdr:col>
-      <xdr:colOff>581024</xdr:colOff>
+      <xdr:colOff>581025</xdr:colOff>
       <xdr:row>2</xdr:row>
       <xdr:rowOff>152400</xdr:rowOff>
     </xdr:to>
@@ -913,19 +913,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:R250"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.75" style="7" customWidth="1"/>
-    <col min="2" max="2" width="10.375" customWidth="1"/>
-    <col min="3" max="9" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="11.5" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.5" bestFit="1" customWidth="1"/>
-    <col min="12" max="13" width="10.375" customWidth="1"/>
-    <col min="14" max="14" width="11.5" style="7" customWidth="1"/>
-    <col min="15" max="18" width="11.125" style="10" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="18.77734375" style="7" customWidth="1"/>
+    <col min="2" max="2" width="10.33203125" customWidth="1"/>
+    <col min="3" max="9" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="11.44140625" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.44140625" bestFit="1" customWidth="1"/>
+    <col min="12" max="13" width="10.33203125" customWidth="1"/>
+    <col min="14" max="14" width="11.44140625" style="7" customWidth="1"/>
+    <col min="15" max="18" width="11.109375" style="10" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:18" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -933,7 +933,7 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:18" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:18" ht="18" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
@@ -14291,12 +14291,14 @@
         <v>40595854</v>
       </c>
       <c r="E246" s="6">
-        <v>41534424</v>
+        <v>41787218</v>
       </c>
       <c r="F246" s="6">
-        <v>46422927</v>
-      </c>
-      <c r="G246" s="6"/>
+        <v>49584803</v>
+      </c>
+      <c r="G246" s="6">
+        <v>53250752</v>
+      </c>
       <c r="H246" s="6"/>
       <c r="I246" s="6"/>
       <c r="J246" s="6"/>
@@ -14305,7 +14307,7 @@
       <c r="M246" s="5"/>
       <c r="N246" s="8">
         <f>SUM(B246:M246)</f>
-        <v>189378011</v>
+        <v>246043433</v>
       </c>
       <c r="O246" s="11">
         <f>SUM(B246:D246)</f>
@@ -14313,7 +14315,7 @@
       </c>
       <c r="P246" s="11">
         <f>SUM(E246:G246)</f>
-        <v>87957351</v>
+        <v>144622773</v>
       </c>
       <c r="Q246" s="11">
         <f>SUM(H246:J246)</f>
@@ -14338,12 +14340,14 @@
         <v>6530959</v>
       </c>
       <c r="E247" s="6">
-        <v>6754705</v>
+        <v>6679549</v>
       </c>
       <c r="F247" s="6">
-        <v>8014839</v>
-      </c>
-      <c r="G247" s="6"/>
+        <v>8156442</v>
+      </c>
+      <c r="G247" s="6">
+        <v>8173113</v>
+      </c>
       <c r="H247" s="6"/>
       <c r="I247" s="6"/>
       <c r="J247" s="6"/>
@@ -14352,7 +14356,7 @@
       <c r="M247" s="5"/>
       <c r="N247" s="8">
         <f>SUM(B247:M247)</f>
-        <v>33367428</v>
+        <v>41606988</v>
       </c>
       <c r="O247" s="11">
         <f>SUM(B247:D247)</f>
@@ -14360,7 +14364,7 @@
       </c>
       <c r="P247" s="11">
         <f>SUM(E247:G247)</f>
-        <v>14769544</v>
+        <v>23009104</v>
       </c>
       <c r="Q247" s="11">
         <f>SUM(H247:J247)</f>
@@ -14385,12 +14389,14 @@
         <v>4467292</v>
       </c>
       <c r="E248" s="6">
-        <v>4428604</v>
+        <v>4437900</v>
       </c>
       <c r="F248" s="6">
-        <v>4857631</v>
-      </c>
-      <c r="G248" s="6"/>
+        <v>4928460</v>
+      </c>
+      <c r="G248" s="6">
+        <v>5662074</v>
+      </c>
       <c r="H248" s="6"/>
       <c r="I248" s="6"/>
       <c r="J248" s="6"/>
@@ -14399,7 +14405,7 @@
       <c r="M248" s="5"/>
       <c r="N248" s="8">
         <f>SUM(B248:M248)</f>
-        <v>21436254</v>
+        <v>27178453</v>
       </c>
       <c r="O248" s="11">
         <f>SUM(B248:D248)</f>
@@ -14407,7 +14413,7 @@
       </c>
       <c r="P248" s="11">
         <f>SUM(E248:G248)</f>
-        <v>9286235</v>
+        <v>15028434</v>
       </c>
       <c r="Q248" s="11">
         <f>SUM(H248:J248)</f>
@@ -14432,12 +14438,14 @@
         <v>64615492</v>
       </c>
       <c r="E249" s="6">
-        <v>60958983</v>
+        <v>61011203</v>
       </c>
       <c r="F249" s="6">
-        <v>72642332</v>
-      </c>
-      <c r="G249" s="6"/>
+        <v>74821190</v>
+      </c>
+      <c r="G249" s="6">
+        <v>84848976</v>
+      </c>
       <c r="H249" s="6"/>
       <c r="I249" s="6"/>
       <c r="J249" s="6"/>
@@ -14446,7 +14454,7 @@
       <c r="M249" s="5"/>
       <c r="N249" s="8">
         <f>SUM(B249:M249)</f>
-        <v>299978384</v>
+        <v>387058438</v>
       </c>
       <c r="O249" s="11">
         <f>SUM(B249:D249)</f>
@@ -14454,7 +14462,7 @@
       </c>
       <c r="P249" s="11">
         <f>SUM(E249:G249)</f>
-        <v>133601315</v>
+        <v>220681369</v>
       </c>
       <c r="Q249" s="11">
         <f>SUM(H249:J249)</f>
@@ -14479,12 +14487,14 @@
         <v>116209597</v>
       </c>
       <c r="E250" s="6">
-        <v>113676716</v>
+        <v>113915870</v>
       </c>
       <c r="F250" s="6">
-        <v>131937729</v>
-      </c>
-      <c r="G250" s="6"/>
+        <v>137490895</v>
+      </c>
+      <c r="G250" s="6">
+        <v>151934915</v>
+      </c>
       <c r="H250" s="6"/>
       <c r="I250" s="6"/>
       <c r="J250" s="6"/>
@@ -14493,7 +14503,7 @@
       <c r="M250" s="5"/>
       <c r="N250" s="8">
         <f>SUM(N246:N249)</f>
-        <v>544160077</v>
+        <v>701887312</v>
       </c>
       <c r="O250" s="11">
         <f>SUM(B250:D250)</f>
@@ -14501,7 +14511,7 @@
       </c>
       <c r="P250" s="11">
         <f>SUM(E250:G250)</f>
-        <v>245614445</v>
+        <v>403341680</v>
       </c>
       <c r="Q250" s="11">
         <f>SUM(H250:J250)</f>
@@ -14596,18 +14606,20 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:M250"/>
-  <sheetFormatPr defaultRowHeight="13.8" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="13" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="18.375" customWidth="1"/>
-    <col min="2" max="4" width="10.375" customWidth="1"/>
-    <col min="5" max="5" width="11.125" bestFit="1" customWidth="1"/>
-    <col min="6" max="13" width="10.375" customWidth="1"/>
-    <col min="14" max="17" width="9.375" customWidth="1"/>
-    <col min="18" max="18" width="3.75" customWidth="1"/>
-    <col min="19" max="19" width="5.125" customWidth="1"/>
+    <col min="1" max="1" width="18.33203125" customWidth="1"/>
+    <col min="2" max="4" width="10.33203125" customWidth="1"/>
+    <col min="5" max="5" width="11.109375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11" customWidth="1"/>
+    <col min="7" max="7" width="11.77734375" customWidth="1"/>
+    <col min="8" max="13" width="10.33203125" customWidth="1"/>
+    <col min="14" max="17" width="9.33203125" customWidth="1"/>
+    <col min="18" max="18" width="3.77734375" customWidth="1"/>
+    <col min="19" max="19" width="5.109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:13" ht="18" x14ac:dyDescent="0.4">
       <c r="A1" s="1" t="s">
         <v>26</v>
       </c>
@@ -14615,14 +14627,14 @@
         <v>25</v>
       </c>
     </row>
-    <row r="2" spans="1:13" ht="17.399999999999999" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:13" ht="18" x14ac:dyDescent="0.4">
       <c r="A2" s="3" t="s">
         <v>27</v>
       </c>
       <c r="F2" s="1"/>
       <c r="M2" s="2"/>
     </row>
-    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:13" ht="18.75" customHeight="1" x14ac:dyDescent="0.4">
       <c r="A3" t="s">
         <v>24</v>
       </c>
@@ -24724,15 +24736,15 @@
       </c>
       <c r="E246" s="5">
         <f>IF('Monthly Data'!E246=0,0,AVERAGE('Monthly Data'!C246,'Monthly Data'!D246,'Monthly Data'!E246))</f>
-        <v>39443344.333333336</v>
+        <v>39527609</v>
       </c>
       <c r="F246" s="5">
         <f>IF('Monthly Data'!F246=0,0,AVERAGE('Monthly Data'!D246,'Monthly Data'!E246,'Monthly Data'!F246))</f>
-        <v>42851068.333333336</v>
+        <v>43989291.666666664</v>
       </c>
       <c r="G246" s="5">
         <f>IF('Monthly Data'!G246=0,0,AVERAGE('Monthly Data'!E246,'Monthly Data'!F246,'Monthly Data'!G246))</f>
-        <v>0</v>
+        <v>48207591</v>
       </c>
       <c r="H246" s="5">
         <f>IF('Monthly Data'!H246=0,0,AVERAGE('Monthly Data'!F246,'Monthly Data'!G246,'Monthly Data'!H246))</f>
@@ -24777,15 +24789,15 @@
       </c>
       <c r="E247" s="5">
         <f>IF('Monthly Data'!E247=0,0,AVERAGE('Monthly Data'!C247,'Monthly Data'!D247,'Monthly Data'!E247))</f>
-        <v>6615398.666666667</v>
+        <v>6590346.666666667</v>
       </c>
       <c r="F247" s="5">
         <f>IF('Monthly Data'!F247=0,0,AVERAGE('Monthly Data'!D247,'Monthly Data'!E247,'Monthly Data'!F247))</f>
-        <v>7100167.666666667</v>
+        <v>7122316.666666667</v>
       </c>
       <c r="G247" s="5">
         <f>IF('Monthly Data'!G247=0,0,AVERAGE('Monthly Data'!E247,'Monthly Data'!F247,'Monthly Data'!G247))</f>
-        <v>0</v>
+        <v>7669701.333333333</v>
       </c>
       <c r="H247" s="5">
         <f>IF('Monthly Data'!H247=0,0,AVERAGE('Monthly Data'!F247,'Monthly Data'!G247,'Monthly Data'!H247))</f>
@@ -24830,15 +24842,15 @@
       </c>
       <c r="E248" s="5">
         <f>IF('Monthly Data'!E248=0,0,AVERAGE('Monthly Data'!C248,'Monthly Data'!D248,'Monthly Data'!E248))</f>
-        <v>4309330.333333333</v>
+        <v>4312429</v>
       </c>
       <c r="F248" s="5">
         <f>IF('Monthly Data'!F248=0,0,AVERAGE('Monthly Data'!D248,'Monthly Data'!E248,'Monthly Data'!F248))</f>
-        <v>4584509</v>
+        <v>4611217.333333333</v>
       </c>
       <c r="G248" s="5">
         <f>IF('Monthly Data'!G248=0,0,AVERAGE('Monthly Data'!E248,'Monthly Data'!F248,'Monthly Data'!G248))</f>
-        <v>0</v>
+        <v>5009478</v>
       </c>
       <c r="H248" s="5">
         <f>IF('Monthly Data'!H248=0,0,AVERAGE('Monthly Data'!F248,'Monthly Data'!G248,'Monthly Data'!H248))</f>
@@ -24883,15 +24895,15 @@
       </c>
       <c r="E249" s="5">
         <f>IF('Monthly Data'!E249=0,0,AVERAGE('Monthly Data'!C249,'Monthly Data'!D249,'Monthly Data'!E249))</f>
-        <v>60112433.666666664</v>
+        <v>60129840.333333336</v>
       </c>
       <c r="F249" s="5">
         <f>IF('Monthly Data'!F249=0,0,AVERAGE('Monthly Data'!D249,'Monthly Data'!E249,'Monthly Data'!F249))</f>
-        <v>66072269</v>
+        <v>66815961.666666664</v>
       </c>
       <c r="G249" s="5">
         <f>IF('Monthly Data'!G249=0,0,AVERAGE('Monthly Data'!E249,'Monthly Data'!F249,'Monthly Data'!G249))</f>
-        <v>0</v>
+        <v>73560456.333333328</v>
       </c>
       <c r="H249" s="5">
         <f>IF('Monthly Data'!H249=0,0,AVERAGE('Monthly Data'!F249,'Monthly Data'!G249,'Monthly Data'!H249))</f>
@@ -24936,15 +24948,15 @@
       </c>
       <c r="E250" s="5">
         <f>IF('Monthly Data'!E250=0,0,AVERAGE('Monthly Data'!C250,'Monthly Data'!D250,'Monthly Data'!E250))</f>
-        <v>110480507</v>
+        <v>110560225</v>
       </c>
       <c r="F250" s="5">
         <f>IF('Monthly Data'!F250=0,0,AVERAGE('Monthly Data'!D250,'Monthly Data'!E250,'Monthly Data'!F250))</f>
-        <v>120608014</v>
+        <v>122538787.33333333</v>
       </c>
       <c r="G250" s="5">
         <f>IF('Monthly Data'!G250=0,0,AVERAGE('Monthly Data'!E250,'Monthly Data'!F250,'Monthly Data'!G250))</f>
-        <v>0</v>
+        <v>134447226.66666666</v>
       </c>
       <c r="H250" s="5">
         <f>IF('Monthly Data'!H250=0,0,AVERAGE('Monthly Data'!F250,'Monthly Data'!G250,'Monthly Data'!H250))</f>

</xml_diff>